<commit_message>
London: Spesenaufstellung statt Reisekostenabrechnung
Sascha bezieht von CGT keinen Lohn, sondern stellt Rechnungen. Damit sind
die Positionen weiterberechnete Spesen und gehoeren als Teil des Entgelts
mit 19 Prozent in seine Rechnung, nicht als steuerfreie Erstattung an einen
Arbeitnehmer. Datei entsprechend umgebaut und umbenannt: Anlage zur
Rechnung, 267,98 EUR netto.

Hotel hat die Firma direkt gezahlt und ist aus der Aufstellung raus. Damit
ist kein Feld mehr offen.

Regel zur Umsatzsteuer bei weiterberechneten Spesen in
wissen/reisekosten.md ergaenzt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-weiterbelastung-fluege-holding-an-cgt.xlsx
+++ b/10_Output/2026-10-21-weiterbelastung-fluege-holding-an-cgt.xlsx
@@ -379,88 +379,92 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -719,325 +723,325 @@
   <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="H4" s="2" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="H4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="2"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="9" t="n">
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="10" t="n">
         <v>111.97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="9" t="n">
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="10" t="n">
         <v>89.98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11" t="s">
+      <c r="A17" s="11"/>
+      <c r="B17" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="12" t="n">
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="13" t="n">
         <f aca="false">SUM(I15:I16)</f>
         <v>201.95</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="15" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
     </row>
     <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
     </row>
     <row r="27" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="C27" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="20"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
     </row>
     <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="C28" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>